<commit_message>
added community database and try image
</commit_message>
<xml_diff>
--- a/App/CLI-backend/App/CLI-backend/databases/PostDatabase.xlsx
+++ b/App/CLI-backend/App/CLI-backend/databases/PostDatabase.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>ID</t>
   </si>
@@ -33,6 +33,27 @@
   </si>
   <si>
     <t>NSFW</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>admin</t>
+  </si>
+  <si>
+    <t>das</t>
+  </si>
+  <si>
+    <t>d</t>
+  </si>
+  <si>
+    <t>assets\images\1784571312685_parrots.jpg</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>false</t>
   </si>
 </sst>
 </file>
@@ -77,16 +98,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="2.640625" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="4.63671875" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="4.44140625" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="8.171875" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="9.14453125" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="10.25390625" customWidth="true" bestFit="true"/>
-    <col min="7" max="7" width="5.7734375" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="2.640625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="5.9765625"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="4.44140625"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="8.171875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="35.76171875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="10.25390625"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="5.7734375"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -112,6 +133,29 @@
         <v>6</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="F2" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="G2" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>